<commit_message>
docs: booking API 명세서 추가, booking postman json 추가
</commit_message>
<xml_diff>
--- a/docs/phi/API 명세서.xlsx
+++ b/docs/phi/API 명세서.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\KDT\git\mjc_b-hotel-reservation\docs\phi\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PHI\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48EC98DE-EB3C-4A0F-B92B-9B23EF2676DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91115BB5-6C6C-4F4B-9AC2-36F31D9700B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2242" yWindow="322" windowWidth="16485" windowHeight="12136" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="90" yWindow="465" windowWidth="21510" windowHeight="12135" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="29">
   <si>
     <t>화면ID</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -76,6 +76,70 @@
   </si>
   <si>
     <t>회원가입</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>B001</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>BookingDto</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>USER</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ResponseEntity&lt;ApiResponse&lt;BookingDto&gt;&gt;</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>B002</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>PATCH</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>GET</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Long userId</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ResponseEntity&lt;ApiResponse&lt;List&lt;BookingDto&gt;&gt;&gt;</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>/api/bookings/insert</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>/api/bookings/{userId}</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>/api/bookings/cancel/{bookingId}</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Long bookingId</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>예약 취소</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>모든 예약 내역 검색</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>객실 1개 예약</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -401,11 +465,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr defaultRowHeight="16.899999999999999" x14ac:dyDescent="0.6"/>
   <cols>
     <col min="1" max="1" width="1.5625" customWidth="1"/>
-    <col min="3" max="3" width="15.5625" customWidth="1"/>
+    <col min="2" max="3" width="15.5625" customWidth="1"/>
     <col min="4" max="5" width="20.5625" customWidth="1"/>
     <col min="6" max="6" width="15.5625" customWidth="1"/>
     <col min="7" max="8" width="20.5625" customWidth="1"/>
@@ -457,6 +521,75 @@
         <v>1</v>
       </c>
     </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.6">
+      <c r="B3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D3" t="s">
+        <v>22</v>
+      </c>
+      <c r="E3" t="s">
+        <v>14</v>
+      </c>
+      <c r="F3" t="s">
+        <v>15</v>
+      </c>
+      <c r="G3" t="s">
+        <v>28</v>
+      </c>
+      <c r="H3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.6">
+      <c r="B4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D4" t="s">
+        <v>23</v>
+      </c>
+      <c r="E4" t="s">
+        <v>20</v>
+      </c>
+      <c r="F4" t="s">
+        <v>15</v>
+      </c>
+      <c r="G4" t="s">
+        <v>27</v>
+      </c>
+      <c r="H4" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.6">
+      <c r="B5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D5" t="s">
+        <v>24</v>
+      </c>
+      <c r="E5" t="s">
+        <v>25</v>
+      </c>
+      <c r="F5" t="s">
+        <v>15</v>
+      </c>
+      <c r="G5" t="s">
+        <v>26</v>
+      </c>
+      <c r="H5" t="s">
+        <v>16</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>